<commit_message>
customertype and paymentmode by COUNTIF AND COUNTIFS
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Documents\Advance Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDAFBFBB-CDA1-44BF-9ED4-7E3995134E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{028FA3A7-76DB-4B99-953D-D4DFB23D465A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,11 @@
   </sheets>
   <definedNames>
     <definedName name="Cat">Dmart_Sales_Data[Category]</definedName>
+    <definedName name="CustomerT">Sheet1!$T$21</definedName>
     <definedName name="Discount">Dmart_Sales_Data[discount]</definedName>
+    <definedName name="Orders">Dmart_Sales_Data[[#Headers],[Column1]]</definedName>
+    <definedName name="Payment">Dmart_Sales_Data[[#Headers],[payment_mode]]</definedName>
+    <definedName name="RE">Dmart_Sales_Data[[#Headers],[Updated_Region]]</definedName>
     <definedName name="Regions">Dmart_Sales_Data[Region]</definedName>
     <definedName name="Saless">Dmart_Sales_Data[sales]</definedName>
   </definedNames>
@@ -66,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4673" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4683" uniqueCount="665">
   <si>
     <t>Column1</t>
   </si>
@@ -2031,6 +2035,36 @@
   </si>
   <si>
     <t>NO Category Sales</t>
+  </si>
+  <si>
+    <t>Total Orders</t>
+  </si>
+  <si>
+    <t>TRANSACTIONS DONE BY CARD</t>
+  </si>
+  <si>
+    <t>TRANSACTIONS DONE BY UPI</t>
+  </si>
+  <si>
+    <t>TRANSACTIONS DONE BY CASH</t>
+  </si>
+  <si>
+    <t>No.OF Transaction having Sales value&gt;4000</t>
+  </si>
+  <si>
+    <t>No.OF Transaction having Sales value&gt;4000 but region NORTH</t>
+  </si>
+  <si>
+    <t>No.OF Transaction having Sales value&gt;4000 but region EAST</t>
+  </si>
+  <si>
+    <t>No.OF Transaction having Sales value&gt;4000 but region WEST</t>
+  </si>
+  <si>
+    <t>No.OF Transaction having Sales value&gt;4000 but region SOUTH</t>
+  </si>
+  <si>
+    <t>Count of sales for custType Member and Payment UPI Or CARD</t>
   </si>
 </sst>
 </file>
@@ -2039,9 +2073,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
-    <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2180,6 +2214,19 @@
       <sz val="11"/>
       <color theme="8" tint="-0.249977111117893"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -2336,7 +2383,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2414,45 +2461,23 @@
     <xf numFmtId="0" fontId="18" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="31">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF212529"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF4F4F4"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2520,6 +2545,31 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF4F4F4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF212529"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
@@ -2546,7 +2596,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0.00"/>
+      <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2554,56 +2604,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF212529"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF4F4F4"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12.3"/>
-        <color rgb="FF333333"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFD8D8D8"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2657,17 +2657,67 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <top style="medium">
+          <color rgb="FFA4A4A4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF212529"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF4F4F4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="medium">
           <color rgb="FFA4A4A4"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color rgb="FFA4A4A4"/>
-        </top>
-      </border>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12.3"/>
+        <color rgb="FF333333"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD8D8D8"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -3077,16 +3127,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{97762E84-48E0-42EB-A297-65A392978E80}" name="Table3" displayName="Table3" ref="D2:H9" totalsRowShown="0" headerRowDxfId="9" dataDxfId="10" headerRowBorderDxfId="12" tableBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{97762E84-48E0-42EB-A297-65A392978E80}" name="Table3" displayName="Table3" ref="D2:H9" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10">
   <autoFilter ref="D2:H9" xr:uid="{97762E84-48E0-42EB-A297-65A392978E80}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{04D31066-1E3C-4184-8E77-38D4373C09E3}" name="Category" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{04D31066-1E3C-4184-8E77-38D4373C09E3}" name="Category" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{B4ED27EB-1280-4573-825E-1FAE5F5D223B}" name="Food" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{84AD34BF-6AB9-4F43-8B3A-631B286FA799}" name="Sales" dataDxfId="7"/>
     <tableColumn id="4" xr3:uid="{B054319D-30B4-4366-9FD9-682FFDDFADA1}" name="FRUITSALES" dataDxfId="6">
       <calculatedColumnFormula>SUMIF(D3:D9,"=Fruits",F3:F9)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DE0E48A9-2D8C-40D1-8D6A-E2D571049241}" name="Column1" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{DE0E48A9-2D8C-40D1-8D6A-E2D571049241}" name="Column1" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3311,8 +3361,9 @@
     <col min="16" max="16" width="8.6640625" customWidth="1"/>
     <col min="17" max="17" width="12.88671875" customWidth="1"/>
     <col min="18" max="18" width="8.6640625" customWidth="1"/>
-    <col min="19" max="19" width="44.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="8.6640625" customWidth="1"/>
+    <col min="19" max="19" width="63.109375" customWidth="1"/>
+    <col min="20" max="20" width="19.44140625" customWidth="1"/>
+    <col min="21" max="23" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -3502,7 +3553,7 @@
         <v>no</v>
       </c>
       <c r="R3" s="5"/>
-      <c r="S3" s="49">
+      <c r="S3" s="48">
         <f>SUMIF(M2:M500,"=UPI",E2:E500)</f>
         <v>386412.25</v>
       </c>
@@ -3639,7 +3690,7 @@
         <v>yes</v>
       </c>
       <c r="R5" s="5"/>
-      <c r="S5" s="49">
+      <c r="S5" s="48">
         <f>SUMIF(M2:M500,"=Cash",E2:E500)</f>
         <v>522964.3</v>
       </c>
@@ -3776,7 +3827,7 @@
         <v>yes</v>
       </c>
       <c r="R7" s="5"/>
-      <c r="S7" s="49">
+      <c r="S7" s="48">
         <f>SUMIF(M2:M500,"=Card",E2:E500)</f>
         <v>413292.63999999996</v>
       </c>
@@ -3977,7 +4028,7 @@
         <v>no</v>
       </c>
       <c r="R10" s="5"/>
-      <c r="S10" s="50" cm="1">
+      <c r="S10" s="49" cm="1">
         <f t="array" ref="S10">SUMIFS(Saless,Cat,"Electronics",Regions,"North",Discount,"&gt;0.40")</f>
         <v>36091.269999999997</v>
       </c>
@@ -4112,8 +4163,13 @@
         <v>no</v>
       </c>
       <c r="R12" s="5"/>
-      <c r="S12" s="5"/>
-      <c r="T12" s="5"/>
+      <c r="S12" s="44" t="s">
+        <v>655</v>
+      </c>
+      <c r="T12" s="52">
+        <f>COUNT(Saless)</f>
+        <v>498</v>
+      </c>
       <c r="U12" s="5"/>
       <c r="V12" s="5"/>
       <c r="W12" s="5"/>
@@ -4178,8 +4234,13 @@
         <v>no</v>
       </c>
       <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
-      <c r="T13" s="5"/>
+      <c r="S13" s="44" t="s">
+        <v>657</v>
+      </c>
+      <c r="T13" s="52">
+        <f>COUNTIF(Dmart_Sales_Data[payment_mode],"=UPI")</f>
+        <v>149</v>
+      </c>
       <c r="U13" s="5"/>
       <c r="V13" s="5"/>
       <c r="W13" s="5"/>
@@ -4244,8 +4305,13 @@
         <v>no</v>
       </c>
       <c r="R14" s="5"/>
-      <c r="S14" s="5"/>
-      <c r="T14" s="5"/>
+      <c r="S14" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="T14" s="52">
+        <f>COUNTIF(Dmart_Sales_Data[payment_mode],"=CARD")</f>
+        <v>164</v>
+      </c>
       <c r="U14" s="5"/>
       <c r="V14" s="5"/>
       <c r="W14" s="5"/>
@@ -4310,8 +4376,13 @@
         <v>no</v>
       </c>
       <c r="R15" s="5"/>
-      <c r="S15" s="5"/>
-      <c r="T15" s="22"/>
+      <c r="S15" s="44" t="s">
+        <v>658</v>
+      </c>
+      <c r="T15" s="52">
+        <f>COUNTIF(Dmart_Sales_Data[payment_mode],"=Cash")</f>
+        <v>185</v>
+      </c>
       <c r="U15" s="22"/>
       <c r="V15" s="5"/>
       <c r="W15" s="5"/>
@@ -4376,8 +4447,13 @@
         <v>no</v>
       </c>
       <c r="R16" s="5"/>
-      <c r="S16" s="5"/>
-      <c r="T16" s="22"/>
+      <c r="S16" s="44" t="s">
+        <v>659</v>
+      </c>
+      <c r="T16" s="53" cm="1">
+        <f t="array" ref="T16">COUNTIF(Saless,"&gt;4000")</f>
+        <v>115</v>
+      </c>
       <c r="U16" s="22"/>
       <c r="V16" s="5"/>
       <c r="W16" s="5"/>
@@ -4442,8 +4518,13 @@
         <v>yes</v>
       </c>
       <c r="R17" s="5"/>
-      <c r="S17" s="5"/>
-      <c r="T17" s="22"/>
+      <c r="S17" s="44" t="s">
+        <v>660</v>
+      </c>
+      <c r="T17" s="53" cm="1">
+        <f t="array" ref="T17">COUNTIFS(Saless,"&gt;4000",Regions,"=North")</f>
+        <v>32</v>
+      </c>
       <c r="U17" s="22"/>
       <c r="V17" s="5"/>
       <c r="W17" s="5"/>
@@ -4508,8 +4589,13 @@
         <v>yes</v>
       </c>
       <c r="R18" s="5"/>
-      <c r="S18" s="5"/>
-      <c r="T18" s="22"/>
+      <c r="S18" s="44" t="s">
+        <v>661</v>
+      </c>
+      <c r="T18" s="53" cm="1">
+        <f t="array" ref="T18">COUNTIFS(Saless,"&gt;4000",Regions,"=East")</f>
+        <v>29</v>
+      </c>
       <c r="U18" s="22"/>
       <c r="V18" s="5"/>
       <c r="W18" s="5"/>
@@ -4574,8 +4660,13 @@
         <v>no</v>
       </c>
       <c r="R19" s="5"/>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
+      <c r="S19" s="44" t="s">
+        <v>662</v>
+      </c>
+      <c r="T19" s="53" cm="1">
+        <f t="array" ref="T19">COUNTIFS(Saless,"&gt;4000",Regions,"=West")</f>
+        <v>27</v>
+      </c>
       <c r="U19" s="5"/>
       <c r="V19" s="5"/>
       <c r="W19" s="5"/>
@@ -4640,8 +4731,13 @@
         <v>yes</v>
       </c>
       <c r="R20" s="5"/>
-      <c r="S20" s="5"/>
-      <c r="T20" s="5"/>
+      <c r="S20" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="T20" s="53" cm="1">
+        <f t="array" ref="T20">COUNTIFS(Saless,"&gt;4000",Regions,"=South")</f>
+        <v>27</v>
+      </c>
       <c r="U20" s="5"/>
       <c r="V20" s="5"/>
       <c r="W20" s="5"/>
@@ -4706,7 +4802,7 @@
         <v>no</v>
       </c>
       <c r="R21" s="5"/>
-      <c r="S21" s="5"/>
+      <c r="S21" s="50"/>
       <c r="T21" s="5"/>
       <c r="U21" s="5"/>
       <c r="V21" s="5"/>
@@ -4772,8 +4868,13 @@
         <v>no</v>
       </c>
       <c r="R22" s="5"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="5"/>
+      <c r="S22" s="44" t="s">
+        <v>664</v>
+      </c>
+      <c r="T22" s="51">
+        <f>COUNTIFS(Dmart_Sales_Data[customer_type],"Member",Dmart_Sales_Data[payment_mode],"UPI")+COUNTIFS(Dmart_Sales_Data[customer_type],"Member",Dmart_Sales_Data[payment_mode],"Card")</f>
+        <v>97</v>
+      </c>
       <c r="U22" s="5"/>
       <c r="V22" s="5"/>
       <c r="W22" s="5"/>
@@ -48793,8 +48894,8 @@
   </sheetData>
   <phoneticPr fontId="9" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576 F1:F499">
-    <cfRule type="top10" dxfId="5" priority="2" bottom="1" rank="10"/>
-    <cfRule type="top10" dxfId="4" priority="3" rank="10"/>
+    <cfRule type="top10" dxfId="4" priority="2" bottom="1" rank="10"/>
+    <cfRule type="top10" dxfId="3" priority="3" rank="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F500:F1048576 G1:G499">
     <cfRule type="colorScale" priority="4">
@@ -48809,7 +48910,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:H499 G500:G1048576">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -49251,7 +49352,7 @@
       <c r="F4" s="47">
         <v>30</v>
       </c>
-      <c r="G4" s="48">
+      <c r="G4" s="45">
         <f>SUMIF(D3:D9,"",F3:F9)</f>
         <v>430</v>
       </c>
@@ -49972,10 +50073,10 @@
   </sortState>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="E2:E9">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>50000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>50000</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>